<commit_message>
ensured that the best individual is kept during subsequent genetic drifts
</commit_message>
<xml_diff>
--- a/Results/genetic_algorithm_run_toy_final_run_4.xlsx
+++ b/Results/genetic_algorithm_run_toy_final_run_4.xlsx
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>162.605403005979</v>
+        <v>213.9923308535895</v>
       </c>
     </row>
     <row r="3">
@@ -651,18 +651,18 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>363.8871461608601</v>
+        <v>399.4195129692951</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -671,18 +671,18 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>17.25269562230277</v>
+        <v>390.4187292100506</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>358.6385762963183</v>
+        <v>16.17332925429928</v>
       </c>
     </row>
   </sheetData>
@@ -727,11 +727,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.8777071028839398</v>
+        <v>0.8774400720735906</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>59.55322990273864,107.65966448874083,551.0921340283301,0.05688067038827351</t>
+          <t>213.9923308535895,390.4187292100506,16.173329254299276,399.41951296929506</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -740,24 +740,24 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.8777071028839398</v>
+        <v>0.8504657649377579</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>162.60540300597896,363.88714616086014,358.6385762963183,17.25269562230277</t>
+          <t>248.0064906661697,390.4187292100506,8.554417902049634,399.41951296929506</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.8765242742547958</v>
+        <v>0.8504657649377579</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>49.549195505364835,396.4917093252266,551.0921340283301,0.11017062035275867</t>
+          <t>217.86405256160322,380.4788632132192,3.73684810511528,1306.1766938947394</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -766,24 +766,24 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.8765242742547958</v>
+        <v>0.8225930763281127</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>102.70684440095305,565.9655565465118,308.20905286337745,28.950426718648586</t>
+          <t>4.6160255950100675,362.7984951588238,138.8888888888889,349.9513879796227</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.8765242742547958</v>
+        <v>0.8225930763281127</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>44.152356076935426,208.52307018764822,406.71669225682626,17.25269562230277</t>
+          <t>4.6160255950100675,968.360250424671,30.800188639092802,349.9513879796227</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -792,63 +792,63 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.8760690602685923</v>
+        <v>0.8225930763281127</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>150.02896765889494,320.8719251415746,276.9022844467214,20.296113621893195</t>
+          <t>243.8079451658561,362.7984951588238,4.620275360414157,891.6897557532476</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.8760690602685923</v>
+        <v>0.8225930763281127</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>150.02896765889494,287.46805857860113,526.9380291508675,10.333006819985213</t>
+          <t>227.52364279579984,968.360250424671,30.800188639092802,349.9513879796227</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.8673177979901516</v>
+        <v>0.8112979457764669</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>113.08915797882769,247.7429227053049,358.6385762963183,33.88778084970793</t>
+          <t>13.8683042179023,584.1982275801909,30.800188639092802,399.41951296929506</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.8673177979901516</v>
+        <v>0.8112979457764669</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>161.07188887363685,208.52307018764822,276.9022844467214,17.440311121371057</t>
+          <t>381.4655309792161,57.93160737632219,10.007147774548855,372.7416780149505</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.8673177979901516</v>
+        <v>0.8112979457764669</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>101.6019675592549,247.7429227053049,276.9022844467214,10.112537911608374</t>
+          <t>243.8079451658561,362.7984951588238,4.620275360414157,349.9513879796227</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -857,132 +857,132 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.8673177979901516</v>
+        <v>0.8112979457764669</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>98.6130249701584,3.0080849114534174,198.34738818592007,17.25269562230277</t>
+          <t>213.9923308535895,390.4187292100506,16.173329254299276,399.41951296929506</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.8673177979901516</v>
+        <v>0.5252676863143443</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>161.07188887363685,208.52307018764822,135.0395642676013,17.25269562230277</t>
+          <t>243.8079451658561,362.7984951588238,121.90397258292803,349.9513879796227</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.763698115252007</v>
+        <v>0.5252676863143443</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>101.6019675592549,287.46805857860113,526.9380291508675,17.25269562230277</t>
+          <t>243.8079451658561,362.7984951588238,138.8888888888889,349.9513879796227</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.763698115252007</v>
+        <v>0.5252676863143443</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>161.07188887363685,247.7429227053049,408.88345842026087,17.25269562230277</t>
+          <t>213.9923308535895,364.3420702518506,121.90397258292803,399.41951296929506</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.763698115252007</v>
+        <v>0.5252676863143443</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>101.6019675592549,247.7429227053049,233.06625216288137,8.413785765373824</t>
+          <t>243.8079451658561,1222.732721524859,138.8888888888889,349.9513879796227</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.763698115252007</v>
+        <v>0.5252676863143443</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>101.6019675592549,247.7429227053049,276.9022844467214,17.25269562230277</t>
+          <t>734.2629847305889,440.319874294407,138.8888888888889,349.9513879796227</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.763698115252007</v>
+        <v>0.5252676863143443</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>50.68097427002624,247.7429227053049,276.9022844467214,22.352417793109247</t>
+          <t>243.8079451658561,362.7984951588238,138.8888888888889,349.9513879796227</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.763698115252007</v>
+        <v>0.5252676863143443</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>113.08915797882769,133.30675605412532,276.9022844467214,26.679331287547576</t>
+          <t>243.8079451658561,690.9067337450248,138.8888888888889,349.9513879796227</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.6359937657526964</v>
+        <v>0.5252676863143443</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>294.6872122730902,247.7429227053049,438.9794318032947,10.112537911608374</t>
+          <t>324.9219909789968,440.319874294407,189.28304798637384,35.244399248027285</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.6359937657526964</v>
+        <v>-1.374864973343592</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>221.5379453519592,565.9655565465118,503.8894243724292,28.959566211312993</t>
+          <t>243.8079451658561,12.068848425439066,138.8888888888889,349.9513879796227</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1026,7 +1026,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1038,7 +1038,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E5</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1050,7 +1050,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>